<commit_message>
Rename landing page entry to index
</commit_message>
<xml_diff>
--- a/outputs/youdefine-sales/YouDefine-Sales.xlsx
+++ b/outputs/youdefine-sales/YouDefine-Sales.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="medipark_leads" sheetId="1" r:id="R6d07f33bfc144cb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정_가이드" sheetId="2" r:id="Raa5a9e62f7de40f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="medipark_leads" sheetId="1" r:id="Rbc0a6ca29bf84212"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정_가이드" sheetId="2" r:id="R136d4ca5c1e54126"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4010,7 +4010,7 @@
         <x:v>랜딩 연결 위치</x:v>
       </x:c>
       <x:c r="B9" s="27" t="str">
-        <x:v>medipark_landing_form_example.html의 APPS_SCRIPT_URL</x:v>
+        <x:v>index.html의 APPS_SCRIPT_URL</x:v>
       </x:c>
     </x:row>
     <x:row r="10">

</xml_diff>